<commit_message>
Bug fix to correct double counting in crude oil production/import/export balancing
</commit_message>
<xml_diff>
--- a/InputData/fuels/PoFDCtAE/Perc of Fuel Demand Changes that Affect Exports.xlsx
+++ b/InputData/fuels/PoFDCtAE/Perc of Fuel Demand Changes that Affect Exports.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-us\InputData\fuels\PoFDCtAE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\fuels\PoFDCtAE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39172FEF-DF46-4438-98F5-4879A2699F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76634699-1010-4FD5-94BB-F02ABA520CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19305" yWindow="-5760" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -434,7 +434,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -458,9 +458,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -783,323 +780,323 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H74"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="87.54296875" customWidth="1"/>
+    <col min="2" max="2" width="87.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>2018</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B12" s="24" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="23" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B13" s="25" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="24" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" s="29" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="26"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B47" s="25"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A57" s="12" t="s">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="13"/>
-      <c r="H57" s="13"/>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>62</v>
       </c>
@@ -1119,83 +1116,83 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.1796875" customWidth="1"/>
-    <col min="2" max="5" width="15.453125" customWidth="1"/>
-    <col min="6" max="6" width="12.81640625" customWidth="1"/>
-    <col min="7" max="7" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="100.7265625" customWidth="1"/>
+    <col min="1" max="1" width="44.140625" customWidth="1"/>
+    <col min="2" max="5" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="100.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="15"/>
-      <c r="H2" s="27" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="14"/>
+      <c r="H2" s="26" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>76</v>
       </c>
       <c r="H3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="21"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="20"/>
       <c r="H4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="21">
         <v>1.3864106347E+16</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="21">
         <v>117950568000000</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="21">
         <v>1906867516000000</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="21">
         <v>1.2075189399E+16</v>
       </c>
       <c r="F5" t="s">
@@ -1205,20 +1202,20 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="21">
         <v>3.5682777E+16</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="21">
         <v>2798295000000000</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="21">
         <v>6809672000000000</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="21">
         <v>3.1671400000000004E+16</v>
       </c>
       <c r="F6" t="s">
@@ -1228,20 +1225,20 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>78</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="21">
         <v>540000000000000</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="21">
         <v>7200000000000000</v>
       </c>
-      <c r="D7" s="22">
-        <v>0</v>
-      </c>
-      <c r="E7" s="22">
+      <c r="D7" s="21">
+        <v>0</v>
+      </c>
+      <c r="E7" s="21">
         <v>7740000000000000</v>
       </c>
       <c r="F7" t="s">
@@ -1251,293 +1248,293 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="21"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
       <c r="H8" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="21"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="20"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="21"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="20"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="21">
         <v>166043036334000</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="21">
         <v>5522103312930.1787</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="21">
         <v>124444981024000</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="19">
         <v>47120158622930.172</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="26" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="21">
         <v>1.8360236509349E+16</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="21">
         <v>59529362424000</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="21">
         <v>1381557079413000</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="19">
         <v>1.703820879236E+16</v>
       </c>
       <c r="F12" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="26" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="21">
         <v>1.0682345175E+16</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="21">
         <v>320229375000000</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="21">
         <v>2936702875000000</v>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="19">
         <v>8065871675000000</v>
       </c>
       <c r="F13" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="21">
         <v>1515620096655000</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="21">
         <v>7285809312000</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="21">
         <v>132183114996000</v>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="19">
         <v>1390722790971000</v>
       </c>
       <c r="F14" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="22">
+      <c r="B15" s="21">
         <v>203604487000000</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="21">
         <v>74398997000000</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="21">
         <v>11939852000000</v>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="19">
         <v>266063632000000</v>
       </c>
       <c r="F15" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="26" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="22">
+      <c r="B16" s="21">
         <v>3537592380000000</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="21">
         <v>338510340000000</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="21">
         <v>393656760000000</v>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="19">
         <v>3482445960000000</v>
       </c>
       <c r="F16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="21"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="20"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="21"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="22">
+      <c r="B19" s="21">
         <v>906213062527442.13</v>
       </c>
-      <c r="C19" s="22">
-        <v>0</v>
-      </c>
-      <c r="D19" s="22">
-        <v>0</v>
-      </c>
-      <c r="E19" s="20">
+      <c r="C19" s="21">
+        <v>0</v>
+      </c>
+      <c r="D19" s="21">
+        <v>0</v>
+      </c>
+      <c r="E19" s="19">
         <v>906213062527442.13</v>
       </c>
       <c r="F19" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="21">
         <v>2.3255085897106E+16</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="21">
         <v>1.269962477E+16</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="21">
         <v>6193988558562000</v>
       </c>
-      <c r="E20" s="20">
+      <c r="E20" s="19">
         <v>2.9760722108544E+16</v>
       </c>
       <c r="F20" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="26" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="21">
         <v>979835237000000</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="21">
         <v>433897305000000</v>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="21">
         <v>705652880000000</v>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="19">
         <v>708079662000000</v>
       </c>
       <c r="F21" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="26" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="21">
         <v>4171558240080000</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="21">
         <v>219065893200000</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="21">
         <v>2412911377800000</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="19">
         <v>1977712755480000</v>
       </c>
       <c r="F22" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="21">
         <v>3564295858911020.5</v>
       </c>
-      <c r="C23" s="22">
-        <v>0</v>
-      </c>
-      <c r="D23" s="22">
-        <v>0</v>
-      </c>
-      <c r="E23" s="20">
+      <c r="C23" s="21">
+        <v>0</v>
+      </c>
+      <c r="D23" s="21">
+        <v>0</v>
+      </c>
+      <c r="E23" s="19">
         <v>3564295858911020.5</v>
       </c>
       <c r="F23" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="21">
         <v>8746500000000000</v>
       </c>
-      <c r="C24" s="22">
-        <v>0</v>
-      </c>
-      <c r="D24" s="22">
-        <v>0</v>
-      </c>
-      <c r="E24" s="20">
+      <c r="C24" s="21">
+        <v>0</v>
+      </c>
+      <c r="D24" s="21">
+        <v>0</v>
+      </c>
+      <c r="E24" s="19">
         <v>8746500000000000</v>
       </c>
       <c r="F24" t="s">
@@ -1555,13 +1552,13 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:V22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.7265625" customWidth="1"/>
-    <col min="2" max="22" width="16.54296875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="22" width="16.5703125" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>69</v>
       </c>
@@ -1629,7 +1626,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -1697,14 +1694,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="5">
         <v>0</v>
       </c>
-      <c r="C3" s="28">
+      <c r="C3" s="27">
         <f>'Data from BFPIaE'!D5/'Data from BFPIaE'!B5</f>
         <v>0.13753987947536334</v>
       </c>
@@ -1766,7 +1763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -1776,7 +1773,7 @@
       <c r="C4" s="7">
         <v>0</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="27">
         <f>'Data from BFPIaE'!D6/'Data from BFPIaE'!B6</f>
         <v>0.19083918272392308</v>
       </c>
@@ -1835,7 +1832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -1848,7 +1845,7 @@
       <c r="D5" s="7">
         <v>0</v>
       </c>
-      <c r="E5" s="28">
+      <c r="E5" s="27">
         <f>'Data from BFPIaE'!D7/'Data from BFPIaE'!B7</f>
         <v>0</v>
       </c>
@@ -1904,7 +1901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>36</v>
       </c>
@@ -1972,7 +1969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>37</v>
       </c>
@@ -2040,7 +2037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>38</v>
       </c>
@@ -2108,7 +2105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -2133,7 +2130,7 @@
       <c r="H9" s="5">
         <v>0</v>
       </c>
-      <c r="I9" s="28">
+      <c r="I9" s="27">
         <f>'Data from BFPIaE'!D11/'Data from BFPIaE'!B11</f>
         <v>0.74947425541939383</v>
       </c>
@@ -2177,7 +2174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -2230,9 +2227,8 @@
       <c r="Q10" s="7">
         <v>0</v>
       </c>
-      <c r="R10" s="11">
-        <f>1-J10</f>
-        <v>0.92499594788389039</v>
+      <c r="R10" s="7">
+        <v>0</v>
       </c>
       <c r="S10" s="7">
         <v>0</v>
@@ -2247,7 +2243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -2300,9 +2296,8 @@
       <c r="Q11" s="7">
         <v>0</v>
       </c>
-      <c r="R11" s="11">
-        <f>1-K11</f>
-        <v>0.73308948177042799</v>
+      <c r="R11" s="7">
+        <v>0</v>
       </c>
       <c r="S11" s="7">
         <v>0</v>
@@ -2317,7 +2312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -2351,7 +2346,7 @@
       <c r="K12" s="7">
         <v>0</v>
       </c>
-      <c r="L12" s="28">
+      <c r="L12" s="27">
         <f>'Data from BFPIaE'!D14/'Data from BFPIaE'!B14</f>
         <v>8.7213883800914521E-2</v>
       </c>
@@ -2386,7 +2381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -2423,7 +2418,7 @@
       <c r="L13" s="7">
         <v>0</v>
       </c>
-      <c r="M13" s="28">
+      <c r="M13" s="27">
         <f>'Data from BFPIaE'!D15/'Data from BFPIaE'!B15</f>
         <v>5.8642381491327347E-2</v>
       </c>
@@ -2455,7 +2450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -2508,9 +2503,8 @@
       <c r="Q14" s="7">
         <v>0</v>
       </c>
-      <c r="R14" s="11">
-        <f>1-N14</f>
-        <v>0.89844005991667841</v>
+      <c r="R14" s="7">
+        <v>0</v>
       </c>
       <c r="S14" s="7">
         <v>0</v>
@@ -2525,7 +2519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>45</v>
       </c>
@@ -2593,7 +2587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>46</v>
       </c>
@@ -2661,7 +2655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -2710,7 +2704,7 @@
       <c r="P17" s="5">
         <v>0</v>
       </c>
-      <c r="Q17" s="28">
+      <c r="Q17" s="27">
         <f>'Data from BFPIaE'!D19/'Data from BFPIaE'!B19</f>
         <v>0</v>
       </c>
@@ -2730,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -2798,7 +2792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>49</v>
       </c>
@@ -2850,9 +2844,8 @@
       <c r="Q19" s="7">
         <v>0</v>
       </c>
-      <c r="R19" s="11">
-        <f>1-S19</f>
-        <v>0.50085828893652218</v>
+      <c r="R19" s="7">
+        <v>0</v>
       </c>
       <c r="S19" s="10">
         <f>'Data from BFPIaE'!D21/SUM('Data from BFPIaE'!D21:E21)</f>
@@ -2868,7 +2861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>50</v>
       </c>
@@ -2920,9 +2913,8 @@
       <c r="Q20" s="7">
         <v>0</v>
       </c>
-      <c r="R20" s="11">
-        <f>1-T20</f>
-        <v>0.45044000475680823</v>
+      <c r="R20" s="7">
+        <v>0</v>
       </c>
       <c r="S20" s="7">
         <v>0</v>
@@ -2938,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>51</v>
       </c>
@@ -2999,7 +2991,7 @@
       <c r="T21" s="7">
         <v>0</v>
       </c>
-      <c r="U21" s="28">
+      <c r="U21" s="27">
         <f>'Data from BFPIaE'!D23/'Data from BFPIaE'!B23</f>
         <v>0</v>
       </c>
@@ -3007,7 +2999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>52</v>
       </c>
@@ -3071,7 +3063,7 @@
       <c r="U22" s="7">
         <v>0</v>
       </c>
-      <c r="V22" s="28">
+      <c r="V22" s="27">
         <f>'Data from BFPIaE'!D24/'Data from BFPIaE'!B24</f>
         <v>0</v>
       </c>

</xml_diff>